<commit_message>
updated check list client for normativity
</commit_message>
<xml_diff>
--- a/taller-6/checklist-cliente.xlsx
+++ b/taller-6/checklist-cliente.xlsx
@@ -701,8 +701,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H24"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.28515625" customWidth="1"/>
@@ -1003,103 +1003,103 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="B12" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="C12" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="D12" t="s">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="E12" t="s">
         <v>29</v>
       </c>
       <c r="F12" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="G12" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="H12" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="C13" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="D13" t="s">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="E13" t="s">
         <v>29</v>
       </c>
       <c r="F13" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="G13" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="H13" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="B14" t="s">
-        <v>37</v>
+        <v>63</v>
       </c>
       <c r="C14" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="D14" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="E14" t="s">
-        <v>29</v>
+        <v>66</v>
       </c>
       <c r="F14" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="G14" t="s">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="H14" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="B15" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="C15" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="D15" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="E15" t="s">
         <v>29</v>
       </c>
       <c r="F15" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="G15" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="H15" t="s">
         <v>25</v>
@@ -1107,51 +1107,51 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="B16" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="C16" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="D16" t="s">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="E16" t="s">
         <v>29</v>
       </c>
       <c r="F16" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="G16" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="H16" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="B17" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="C17" t="s">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="D17" t="s">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="E17" t="s">
         <v>66</v>
       </c>
       <c r="F17" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="G17" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="H17" t="s">
         <v>25</v>
@@ -1159,25 +1159,25 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="B18" t="s">
-        <v>63</v>
+        <v>86</v>
       </c>
       <c r="C18" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="D18" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="E18" t="s">
         <v>29</v>
       </c>
       <c r="F18" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="G18" t="s">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="H18" t="s">
         <v>25</v>
@@ -1185,51 +1185,51 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>74</v>
+        <v>91</v>
       </c>
       <c r="B19" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="C19" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="D19" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E19" t="s">
         <v>29</v>
       </c>
       <c r="F19" t="s">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="G19" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="H19" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="B20" t="s">
-        <v>75</v>
+        <v>97</v>
       </c>
       <c r="C20" t="s">
-        <v>81</v>
+        <v>98</v>
       </c>
       <c r="D20" t="s">
-        <v>82</v>
+        <v>99</v>
       </c>
       <c r="E20" t="s">
         <v>66</v>
       </c>
       <c r="F20" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="G20" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="H20" t="s">
         <v>25</v>
@@ -1237,105 +1237,27 @@
     </row>
     <row r="21" spans="1:8">
       <c r="A21" t="s">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="B21" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="C21" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="D21" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="E21" t="s">
-        <v>29</v>
+        <v>66</v>
       </c>
       <c r="F21" t="s">
-        <v>89</v>
+        <v>104</v>
       </c>
       <c r="G21" t="s">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="H21" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8">
-      <c r="A22" t="s">
-        <v>91</v>
-      </c>
-      <c r="B22" t="s">
-        <v>86</v>
-      </c>
-      <c r="C22" t="s">
-        <v>92</v>
-      </c>
-      <c r="D22" t="s">
-        <v>93</v>
-      </c>
-      <c r="E22" t="s">
-        <v>29</v>
-      </c>
-      <c r="F22" t="s">
-        <v>94</v>
-      </c>
-      <c r="G22" t="s">
-        <v>95</v>
-      </c>
-      <c r="H22" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8">
-      <c r="A23" t="s">
-        <v>96</v>
-      </c>
-      <c r="B23" t="s">
-        <v>97</v>
-      </c>
-      <c r="C23" t="s">
-        <v>98</v>
-      </c>
-      <c r="D23" t="s">
-        <v>99</v>
-      </c>
-      <c r="E23" t="s">
-        <v>66</v>
-      </c>
-      <c r="F23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G23" t="s">
-        <v>101</v>
-      </c>
-      <c r="H23" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8">
-      <c r="A24" t="s">
-        <v>102</v>
-      </c>
-      <c r="B24" t="s">
-        <v>97</v>
-      </c>
-      <c r="C24" t="s">
-        <v>103</v>
-      </c>
-      <c r="D24" t="s">
-        <v>99</v>
-      </c>
-      <c r="E24" t="s">
-        <v>66</v>
-      </c>
-      <c r="F24" t="s">
-        <v>104</v>
-      </c>
-      <c r="G24" t="s">
-        <v>105</v>
-      </c>
-      <c r="H24" t="s">
         <v>42</v>
       </c>
     </row>

</xml_diff>